<commit_message>
Input data changed in register
</commit_message>
<xml_diff>
--- a/DEMOWEBSHOP/src/test/resources/TestData/TestData.xlsx
+++ b/DEMOWEBSHOP/src/test/resources/TestData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vithy\Desktop\Expleo\AUTOMATIONPROJECT\DEMOWEBSHOP\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764AEE57-3D8D-468E-A2A4-42E0B54B8A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D32A30-9425-4C82-8E91-666F280D4ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
     <t>murugesan</t>
   </si>
   <si>
-    <t>vithyamurugesan46@gmail.com</t>
+    <t>vithyamurugesan664456@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -441,7 +441,7 @@
     <col min="5" max="5" width="18.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>

</xml_diff>